<commit_message>
Correct Crown CICRA conditions and volatility sequence
</commit_message>
<xml_diff>
--- a/examples/crown-castle-2025/deliverables/workbook.xlsx
+++ b/examples/crown-castle-2025/deliverables/workbook.xlsx
@@ -5685,7 +5685,7 @@
     <t>2025-07-07原发、2025-09-26重发；PDF61–78数字基础设施章，尤其68–71及77</t>
   </si>
   <si>
-    <t>塔资产提供方与移动运营商付塔费不同。波动档要求业务风险、竞争地位及可预测CFO等共同条件，90%/2/3不是租赁收入比例。土地控制、客户质量和网络必要性可以缓释，但不能替代续约及违约压力。</t>
+    <t>塔资产提供方与移动运营商付塔费不同。先检验low，再在low不成立时检验medial，均不成立才用standard。low要求CICRA为1或2、竞争地位至少strong、至少90%可预测CFO；medial要求CICRA为1至3、竞争地位至少satisfactory、至少2/3可预测CFO。两档分别核合同或支持性监管/合同/法律框架条件，low的框架还须已建立，并均要求其他活动不被视为高风险或具有波动性；收入占比不能替代CFO归属。</t>
   </si>
   <si>
     <t>问题</t>
@@ -6070,10 +6070,10 @@
     <t>经营优势能否支持较低现金流波动档？</t>
   </si>
   <si>
-    <t>自有土地覆盖30.26%的塔，贡献42.68%的末季年化毛现金利润。2028续约组年度化租金暴露中AT&amp;T占90.01%，该暴露不代表当年确定损失。长期租赁及续约经济性支持将medial列为待验证候选；若相应条件不满足则检验standard，不能预授low或直接输出等级。</t>
-  </si>
-  <si>
-    <t>租地35年含公司续约权、账内租赁15年、客户当前合同6年/AT&amp;T3年各有不同定义。土地控制和核心市场规模是正面证据，客户集中及DISH违约为反证。S&amp;P数字基础设施章低/中波动要求业务风险、竞争地位及至少90%/2/3可预测CFO等共同条件；收入占比不能替代CFO归属，客户短剩余期也不单独否定支持性框架路径。本案尚未独立完成CICRA、竞争地位、预测CFO及支持债项形成链，保留明确分支，不将保守标签视作已证实分类。</t>
+    <t>自有土地覆盖30.26%的塔，贡献42.68%的末季年化毛现金利润。2028续约组年度化租金暴露中AT&amp;T占90.01%，该暴露不代表当年确定损失。波动档先检验low的全部条件，再在low不成立时检验medial，均不成立才用standard。本案必要因素尚未完成，不给已确认波动档或等级。</t>
+  </si>
+  <si>
+    <t>Q4资料中的租地35年含公司续约权、账内租赁15年、客户合同6年/AT&amp;T3年各有不同定义。low要求CICRA为1或2、竞争地位至少strong、至少90%可预测CFO；可预测性可来自通常约10年剩余期且高度可能按相近条款续约的长期确定合同，或低政治干预风险的已建立支持性监管/合同/法律框架。low不成立时，medial要求CICRA为1至3、竞争地位至少satisfactory、至少2/3可预测CFO，来自续约风险有限或低的确定合同，或低政治干预风险的支持性监管/合同/法律框架。两档均要求其他活动不被视为高风险或具有波动性。收入占比不能替代CFO归属，客户短剩余期不单独否定框架路径；土地控制和核心市场规模是正面证据，客户集中及DISH违约为反证。尚未完成CICRA、竞争地位及前瞻现金归属，后续支持和债项也各有节点，不能把候选或保守标签视作已证分类。</t>
   </si>
   <si>
     <t>E_SP_LAND, E_SP_RENEW, E_SP_SECTORS, E_SP_Q1BILL, C_sp_renew_share</t>

</xml_diff>